<commit_message>
Cập nhật bộ tài liệu NCC GCN theo bản mới trên Drive
- Lưu trình: cột Bộ phận phụ trách chỉ còn Mua hàng / Chất lượng (bỏ Kỹ thuật, KHSX, dòng phê duyệt); chọn NCC do Mua hàng và Kinh doanh (Nhật) quyết định
- Biểu mẫu: Check sheet rút gọn mở rộng 42 hạng mục, có tiêu chí 1 điểm / 2 điểm, tự tính điểm theo nhóm, kết luận và điểm quy đổi sang QLGCN-02
- File 3 đã gộp vào file 2 nên bỏ khỏi thư mục

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XhQjYi47ydaDu3gmrGesYy
</commit_message>
<xml_diff>
--- a/TAI_LIEU_DANH_GIA_NCC_GCN/1.Luu_trinh_QL_NCC Gia cong ngoai.xlsx
+++ b/TAI_LIEU_DANH_GIA_NCC_GCN/1.Luu_trinh_QL_NCC Gia cong ngoai.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D\管理データ\3.購買部\外注管理\TÀI LIỆU CHUẨN ĐÁNH GIÁ QUẢN LÝ NCC GCN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17a6b3fa349d5a38/Desktop/QL GCN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497CEEBC-8AD3-42A6-A701-A8E66A0BB0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{497CEEBC-8AD3-42A6-A701-A8E66A0BB0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F8D308E-5B62-4130-AD91-96579E33E755}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lưu trình (VN)" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="243">
   <si>
     <t>Mã tài liệu</t>
   </si>
@@ -75,7 +75,7 @@
     <t>Lưu đồ</t>
   </si>
   <si>
-    <t xml:space="preserve">Bộ phận phụ trách</t>
+    <t>Bộ phận phụ trách</t>
   </si>
   <si>
     <t>Nội dung thực hiện</t>
@@ -90,7 +90,7 @@
     <t>- Phát sinh nhu cầu NCC mới / linh kiện mới / ủy thác gia công.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng
+    <t>Mua hàng
 Phối hợp: Chất lượng, Kỹ thuật, KHSX, NCC</t>
   </si>
   <si>
@@ -100,32 +100,32 @@
 - Xác nhận NCC cấp 1 có sử dụng NCC cấp 2 không; nếu có, thu thập thông tin NCC cấp 2 (tên, công đoạn, NVL).</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, Chất lượng
+    <t>Mua hàng, Chất lượng
 Phối hợp: Kỹ thuật, NCC
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, NCC
+    <t>Mua hàng, NCC
 Phối hợp: Chất lượng, Kỹ thuật
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Chất lượng, Kỹ thuật, NCC
+    <t>Chất lượng, Kỹ thuật, NCC
 Phối hợp: Mua hàng, KHSX
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, Chất lượng, KHSX, NCC
+    <t>Mua hàng, Chất lượng, KHSX, NCC
 Phối hợp: Kỹ thuật, Sản xuất
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Chất lượng, Kỹ thuật
+    <t>Chất lượng, Kỹ thuật
 Phối hợp: Mua hàng, NCC
 Phê duyệt: Phụ trách GCN, Chất lượng</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, KHSX, NCC
+    <t>Mua hàng, KHSX, NCC
 Phối hợp: Kho</t>
   </si>
   <si>
@@ -138,7 +138,7 @@
 Bảng quản lý giao hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, Chất lượng, NCC
+    <t>Mua hàng, Chất lượng, NCC
 Phối hợp: KHSX</t>
   </si>
   <si>
@@ -151,7 +151,7 @@
 Bảng quản lý giao hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Kho, NCC
+    <t>Kho, NCC
 Phối hợp: Mua hàng</t>
   </si>
   <si>
@@ -163,7 +163,7 @@
 Phiếu nhập kho</t>
   </si>
   <si>
-    <t xml:space="preserve">Chất lượng
+    <t>Chất lượng
 Phối hợp: Mua hàng, Kho</t>
   </si>
   <si>
@@ -175,12 +175,12 @@
 Kết quả kiểm tra</t>
   </si>
   <si>
-    <t xml:space="preserve">Chất lượng, NCC
+    <t>Chất lượng, NCC
 Phối hợp: Mua hàng, Kỹ thuật
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, NCC
+    <t>Mua hàng, NCC
 Phối hợp: Kho, Kế toán</t>
   </si>
   <si>
@@ -192,7 +192,7 @@
 Đề nghị thanh toán</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng, Kỹ thuật, NCC
+    <t>Mua hàng, Kỹ thuật, NCC
 Phối hợp: Chất lượng
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
@@ -202,7 +202,7 @@
 - Thay đổi quan trọng: sản xuất thử và phê duyệt lại (bước 5–6); cập nhật tài liệu sau khi phê duyệt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua hàng
+    <t>Mua hàng
 Phối hợp: Chất lượng, NCC
 Phê duyệt: Quản lý Mua hàng</t>
   </si>
@@ -243,7 +243,7 @@
     <t>フロー</t>
   </si>
   <si>
-    <t xml:space="preserve">担当部署</t>
+    <t>担当部署</t>
   </si>
   <si>
     <t>説明</t>
@@ -258,7 +258,7 @@
     <t>・新規サプライヤー／新規部品／外部委託の需要発生。</t>
   </si>
   <si>
-    <t xml:space="preserve">購買
+    <t>購買
 協力：品質管理、技術、生産管理、仕入先</t>
   </si>
   <si>
@@ -268,32 +268,32 @@
 ・一次仕入先が二次仕入先を使用するか確認し、使用する場合は二次仕入先の情報（社名、工程、材料）を入手する。</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、品質管理
+    <t>購買、品質管理
 協力：技術、仕入先
 承認：購買管理者</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、仕入先
+    <t>購買、仕入先
 協力：品質管理、技術
 承認：購買管理者</t>
   </si>
   <si>
-    <t xml:space="preserve">品質管理、技術、仕入先
+    <t>品質管理、技術、仕入先
 協力：購買、生産管理
 承認：購買管理者</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、品質管理、生産管理、仕入先
+    <t>購買、品質管理、生産管理、仕入先
 協力：技術、製造
 承認：購買管理者</t>
   </si>
   <si>
-    <t xml:space="preserve">品質管理、技術
+    <t>品質管理、技術
 協力：購買、仕入先
 承認：外注担当、品質管理</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、生産管理、仕入先
+    <t>購買、生産管理、仕入先
 協力：倉庫</t>
   </si>
   <si>
@@ -306,7 +306,7 @@
 納期管理表</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、品質管理、仕入先
+    <t>購買、品質管理、仕入先
 協力：生産管理</t>
   </si>
   <si>
@@ -319,7 +319,7 @@
 納期管理表</t>
   </si>
   <si>
-    <t xml:space="preserve">倉庫、仕入先
+    <t>倉庫、仕入先
 協力：購買</t>
   </si>
   <si>
@@ -331,7 +331,7 @@
 入庫伝票</t>
   </si>
   <si>
-    <t xml:space="preserve">品質管理
+    <t>品質管理
 協力：購買、倉庫</t>
   </si>
   <si>
@@ -343,12 +343,12 @@
 検査記録</t>
   </si>
   <si>
-    <t xml:space="preserve">品質管理、仕入先
+    <t>品質管理、仕入先
 協力：購買、技術
 承認：購買管理者</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、仕入先
+    <t>購買、仕入先
 協力：倉庫、経理</t>
   </si>
   <si>
@@ -360,7 +360,7 @@
 支払依頼書</t>
   </si>
   <si>
-    <t xml:space="preserve">購買、技術、仕入先
+    <t>購買、技術、仕入先
 協力：品質管理
 承認：購買管理者</t>
   </si>
@@ -370,7 +370,7 @@
 ・重要な変更は再試作・再承認（手順5～6）を行い、承認後に関連資料を更新する。</t>
   </si>
   <si>
-    <t xml:space="preserve">購買
+    <t>購買
 協力：品質管理、仕入先
 承認：購買管理者</t>
   </si>
@@ -411,7 +411,7 @@
     <t>作成者</t>
   </si>
   <si>
-    <t xml:space="preserve">- Ký hợp đồng khung / hợp đồng gia công trước khi cung cấp bản vẽ, thông số kỹ thuật. Nội dung gồm: giá, thanh toán, giao hàng, trách nhiệm chất lượng, bảo mật thông tin kỹ thuật.
+    <t>- Ký hợp đồng khung / hợp đồng gia công trước khi cung cấp bản vẽ, thông số kỹ thuật. Nội dung gồm: giá, thanh toán, giao hàng, trách nhiệm chất lượng, bảo mật thông tin kỹ thuật.
 - Hợp đồng quy định NCC cấp 1 phải truyền đạt đầy đủ yêu cầu kỹ thuật, NVL, điều kiện SX cho NCC cấp 2 và báo trước mọi thay đổi 4M / thay đổi NCC cấp 2.
 - Cập nhật trạng thái hợp đồng trong [QLGCN-01].</t>
   </si>
@@ -436,7 +436,7 @@
 (Danh sách NCC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hợp đồng
+    <t>Hợp đồng
 QLGCN-01
 (Danh sách NCC)</t>
   </si>
@@ -472,7 +472,7 @@
 (Danh sách NCC)</t>
   </si>
   <si>
-    <t xml:space="preserve">- Đánh giá hiện trường NCC cấp 1 theo Check sheet đánh giá NCC (0–1–2 điểm), gồm cả nhóm hạng mục quản lý NCC cấp 2.
+    <t>- Đánh giá hiện trường NCC cấp 1 theo Check sheet đánh giá NCC (0–1–2 điểm), gồm cả nhóm hạng mục quản lý NCC cấp 2.
 - Tổng hợp điểm theo [QLGCN-02] (thang 100): ≥80 Đạt; 60–79 Đạt có điều kiện (lập CAR, kỳ hạn, hoàn thành trước MP); &lt;60 Không đạt → quay lại bước 1.
 - Quản lý Mua hàng phê duyệt; Mua hàng cập nhật [QLGCN-01].</t>
   </si>
@@ -488,7 +488,7 @@
 - Mỗi giai đoạn phải đạt và được ký xác nhận trên [QLGCN-03] mới chuyển sang giai đoạn tiếp theo; vấn đề phát sinh ghi vào Sổ theo dõi vấn đề [QLGCN-04].</t>
   </si>
   <si>
-    <t xml:space="preserve">- Kiểm tra kích thước, ngoại quan sản phẩm; đánh giá khả năng SX hàng loạt.
+    <t>- Kiểm tra kích thước, ngoại quan sản phẩm; đánh giá khả năng SX hàng loạt.
 - Điều kiện: hoàn thành 100% hạng mục [QLGCN-03], mẫu Mihonki được khách hàng chấp thuận, CAR (nếu có) đã đóng.
 - OK: Phụ trách GCN và Chất lượng phê duyệt SX hàng loạt (MP). NG: thực hiện đối sách, quay lại bước 5.</t>
   </si>
@@ -534,7 +534,7 @@
     <t>QLGCN-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh mục NCC: thông tin liên hệ, mặt hàng, xếp hạng, trạng thái hợp đồng</t>
+    <t>Danh mục NCC: thông tin liên hệ, mặt hàng, xếp hạng, trạng thái hợp đồng</t>
   </si>
   <si>
     <t>Bước 1, 2, 3, 15</t>
@@ -588,11 +588,11 @@
     <t>Bước 14, 15</t>
   </si>
   <si>
-    <t xml:space="preserve">Check sheet đánh giá NCC
+    <t>Check sheet đánh giá NCC
 (file riêng: 3.Check_sheet_danh_gia_NCC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Đánh giá hiện trường hệ thống chất lượng NCC (0–1–2 điểm): dùng sheet Rút gọn 30 hạng mục; bản đầy đủ 50 hạng mục dùng khi cần đánh giá chuyên sâu</t>
+    <t>Đánh giá hiện trường hệ thống chất lượng NCC (0–1–2 điểm): dùng sheet Rút gọn 30 hạng mục; bản đầy đủ 50 hạng mục dùng khi cần đánh giá chuyên sâu</t>
   </si>
   <si>
     <t>Bước 2, 14</t>
@@ -625,7 +625,7 @@
 （サプライヤー一覧）</t>
   </si>
   <si>
-    <t xml:space="preserve">契約書
+    <t>契約書
 QLGCN-01
 （サプライヤー一覧）</t>
   </si>
@@ -661,12 +661,12 @@
 （サプライヤー一覧）</t>
   </si>
   <si>
-    <t xml:space="preserve">・品質システム監査チェックシート（0・1・2点）で一次仕入先の現地監査を行う（二次仕入先管理の項目を含む）。
+    <t>・品質システム監査チェックシート（0・1・2点）で一次仕入先の現地監査を行う（二次仕入先管理の項目を含む）。
 ・QLGCN-02で総合評価（100点換算）：80点以上＝合格、60～79点＝条件付合格（是正要求・期限設定、量産前に完了）、60点未満＝不合格→手順1へ戻る。
 ・購買管理者が承認し、購買がQLGCN-01を更新する。</t>
   </si>
   <si>
-    <t xml:space="preserve">・図面・仕様書を提供する前に取引基本契約／外注契約を締結する（価格、支払、納入、品質責任、技術情報の秘密保持）。
+    <t>・図面・仕様書を提供する前に取引基本契約／外注契約を締結する（価格、支払、納入、品質責任、技術情報の秘密保持）。
 ・一次仕入先が技術要求・材料・製造条件を二次仕入先へ確実に伝達すること、4M変更・二次仕入先変更を事前連絡することを契約に明記する。
 ・QLGCN-01の契約状況を更新する。</t>
   </si>
@@ -682,7 +682,7 @@
 ・各段階はQLGCN-03で合格・確認サインを得てから次段階へ進む。発生した問題は問題管理表（QLGCN-04）に記録する。</t>
   </si>
   <si>
-    <t xml:space="preserve">・製品の寸法・外観を確認し、量産可否を判断する。
+    <t>・製品の寸法・外観を確認し、量産可否を判断する。
 ・条件：QLGCN-03の全項目完了、見本器の顧客承認取得、是正要求（ある場合）の完了。
 ・OK：外注担当と品質管理が量産（MP）を承認する。NG：対策を実施し、手順5へ戻る。</t>
   </si>
@@ -725,7 +725,7 @@
     <t>外注サプライヤー一覧</t>
   </si>
   <si>
-    <t xml:space="preserve">サプライヤー情報（連絡先、品目、ランク、契約状況）の管理</t>
+    <t>サプライヤー情報（連絡先、品目、ランク、契約状況）の管理</t>
   </si>
   <si>
     <t>手順1、2、3、15</t>
@@ -767,11 +767,11 @@
     <t>手順14、15</t>
   </si>
   <si>
-    <t xml:space="preserve">品質システム監査チェックシート
+    <t>品質システム監査チェックシート
 （別ファイル：3.Check_sheet_danh_gia_NCC）</t>
   </si>
   <si>
-    <t xml:space="preserve">仕入先の品質システム現地監査（0・1・2点）：簡易版30項目を使用、詳細監査時は50項目版を使用</t>
+    <t>仕入先の品質システム現地監査（0・1・2点）：簡易版30項目を使用、詳細監査時は50項目版を使用</t>
   </si>
   <si>
     <t>手順2、14</t>
@@ -784,9 +784,6 @@
   </si>
   <si>
     <t>評価者の要件（手順2、14）</t>
-  </si>
-  <si>
-    <t>様式管理番号追記・4項追加</t>
   </si>
   <si>
     <t>Chưa có mã (lấy mã Cty)</t>
@@ -811,19 +808,142 @@
     <t>保管規定に従う</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa đổi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28/09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bỏ ký NDA, chỉ ký hợp đồng; ghi trực tiếp bộ phận phụ trách (bỏ RACI); thay PL bằng Quản lý Mua hàng, phê duyệt MP do Phụ trách GCN và Chất lượng; cập nhật Check sheet rút gọn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">改訂</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDA廃止（契約のみ）、担当部署を直接記載（RACI廃止）、PLを購買管理者に変更、量産承認は外注担当・品質管理、簡易チェックシート追加</t>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng
+Quyết định chọn NCC: Mua hàng, Kinh doanh (Nhật)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kho, Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng, Chất lượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Đánh giá hiện trường NCC cấp 1 theo Check sheet đánh giá NCC (0–1–2 điểm), gồm cả nhóm hạng mục quản lý NCC cấp 2.
+- Tổng hợp điểm theo [QLGCN-02] (thang 100): ≥80 Đạt; 60–79 Đạt có điều kiện (lập CAR, kỳ hạn, hoàn thành trước MP); &lt;60 Không đạt → quay lại bước 1.
+- Mua hàng và Kinh doanh (Nhật) quyết định chọn NCC; Mua hàng cập nhật [QLGCN-01].</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Kiểm tra kích thước, ngoại quan sản phẩm; đánh giá khả năng SX hàng loạt.
+- Điều kiện: hoàn thành 100% hạng mục [QLGCN-03], mẫu Mihonki được khách hàng chấp thuận, CAR (nếu có) đã đóng.
+- OK: Mua hàng và Chất lượng xác nhận chuyển sang SX hàng loạt (MP). NG: thực hiện đối sách, quay lại bước 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Danh mục biểu mẫu áp dụng (bộ biểu mẫu GCN-NCC-01 – file Bieu_mau_Quan_ly_NCC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check sheet đánh giá NCC
+(file Bieu_mau_Quan_ly_NCC, sheet Check sheet rút gọn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đánh giá hiện trường hệ thống chất lượng NCC (0–1–2 điểm, có tiêu chí 1 điểm / 2 điểm cho từng hạng mục, tự tính điểm). Bản đầy đủ 50 hạng mục (sheet 05.01) dùng khi cần đánh giá chuyên sâu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理
+サプライヤー決定：購買、営業（日本人）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">倉庫、購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買、品質管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">購買</t>
+  </si>
+  <si>
+    <t xml:space="preserve">・品質システム監査チェックシート（0・1・2点）で一次仕入先の現地監査を行う（二次仕入先管理の項目を含む）。
+・QLGCN-02で総合評価（100点換算）：80点以上＝合格、60～79点＝条件付合格（是正要求・期限設定、量産前に完了）、60点未満＝不合格→手順1へ戻る。
+・購買と営業（日本人）がサプライヤーを決定し、購買がQLGCN-01を更新する。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">・製品の寸法・外観を確認し、量産可否を判断する。
+・条件：QLGCN-03の全項目完了、見本器の顧客承認取得、是正要求（ある場合）の完了。
+・OK：購買と品質管理が確認し、量産（MP）へ移行する。NG：対策を実施し、手順5へ戻る。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. 関連様式一覧（様式集 GCN-NCC-01：Bieu_mau_Quan_ly_NCC）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">品質システム監査チェックシート
+（Bieu_mau_Quan_ly_NCC内「Check sheet rút gọn」シート）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">仕入先の品質システム現地監査（0・1・2点、項目毎に1点・2点の基準あり、自動計算）。詳細監査時は50項目版（シート05.01）を使用。</t>
   </si>
 </sst>
 </file>
@@ -1058,28 +1178,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1096,17 +1198,29 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1115,8 +1229,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1128,7 +1242,13 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7709,14 +7829,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="22" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
@@ -7728,24 +7848,24 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="20"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
+      <c r="A3" s="33"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
     </row>
     <row r="4" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7754,15 +7874,15 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
     </row>
     <row r="7" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -7770,15 +7890,15 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
     </row>
     <row r="9" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -7795,11 +7915,11 @@
       <c r="C10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
       <c r="G10" s="2" t="s">
         <v>13</v>
       </c>
@@ -7808,13 +7928,13 @@
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
       <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7823,13 +7943,13 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
       <c r="G12" s="14" t="s">
         <v>100</v>
       </c>
@@ -7840,13 +7960,13 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+        <v>203</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
       <c r="G13" s="14" t="s">
         <v>101</v>
       </c>
@@ -7857,13 +7977,13 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="25" t="s">
+        <v>204</v>
+      </c>
+      <c r="D14" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="14" t="s">
         <v>102</v>
       </c>
@@ -7872,9 +7992,9 @@
       <c r="A15" s="1"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
       <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -7887,11 +8007,11 @@
       <c r="C16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="2" t="s">
         <v>13</v>
       </c>
@@ -7900,9 +8020,9 @@
       <c r="A17" s="1"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
       <c r="G17" s="4"/>
     </row>
     <row r="18" spans="1:7" ht="168" customHeight="1" x14ac:dyDescent="0.3">
@@ -7911,13 +8031,13 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
       <c r="G18" s="4" t="s">
         <v>103</v>
       </c>
@@ -7928,13 +8048,13 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="21" t="s">
+        <v>206</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
       <c r="G19" s="4" t="s">
         <v>104</v>
       </c>
@@ -7945,13 +8065,13 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
+        <v>207</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="4" t="s">
         <v>104</v>
       </c>
@@ -7962,13 +8082,13 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D21" s="21" t="s">
+        <v>208</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
       <c r="G21" s="4" t="s">
         <v>25</v>
       </c>
@@ -7977,9 +8097,9 @@
       <c r="A22" s="1"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
       <c r="G22" s="4"/>
     </row>
     <row r="23" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -7992,11 +8112,11 @@
       <c r="C23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="2" t="s">
         <v>13</v>
       </c>
@@ -8005,9 +8125,9 @@
       <c r="A24" s="1"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
       <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8016,13 +8136,13 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D25" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
       <c r="G25" s="4" t="s">
         <v>28</v>
       </c>
@@ -8033,13 +8153,13 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="D26" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="4" t="s">
         <v>31</v>
       </c>
@@ -8050,13 +8170,13 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D27" s="21" t="s">
+        <v>211</v>
+      </c>
+      <c r="D27" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
       <c r="G27" s="4" t="s">
         <v>34</v>
       </c>
@@ -8067,13 +8187,13 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
       <c r="G28" s="4" t="s">
         <v>105</v>
       </c>
@@ -8084,13 +8204,13 @@
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="21" t="s">
+        <v>213</v>
+      </c>
+      <c r="D29" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="4" t="s">
         <v>38</v>
       </c>
@@ -8099,9 +8219,9 @@
       <c r="A30" s="1"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
       <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8114,11 +8234,11 @@
       <c r="C31" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="22" t="s">
+      <c r="D31" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="2" t="s">
         <v>13</v>
       </c>
@@ -8127,9 +8247,9 @@
       <c r="A32" s="1"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
       <c r="G32" s="4"/>
     </row>
     <row r="33" spans="1:7" ht="151.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -8138,13 +8258,13 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D33" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="D33" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
       <c r="G33" s="4" t="s">
         <v>106</v>
       </c>
@@ -8155,13 +8275,13 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="21" t="s">
+        <v>215</v>
+      </c>
+      <c r="D34" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
       <c r="G34" s="4" t="s">
         <v>107</v>
       </c>
@@ -8172,13 +8292,13 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="21" t="s">
+        <v>216</v>
+      </c>
+      <c r="D35" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
       <c r="G35" s="4" t="s">
         <v>108</v>
       </c>
@@ -8189,18 +8309,18 @@
       <c r="C36" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D36" s="25" t="s">
+      <c r="D36" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="4" t="s">
         <v>199</v>
-      </c>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="4" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>116</v>
+        <v>219</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8213,11 +8333,11 @@
       <c r="C38" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D38" s="22" t="s">
+      <c r="D38" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
       <c r="G38" s="2" t="s">
         <v>121</v>
       </c>
@@ -8232,11 +8352,11 @@
       <c r="C39" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
       <c r="G39" s="14" t="s">
         <v>125</v>
       </c>
@@ -8251,11 +8371,11 @@
       <c r="C40" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
       <c r="G40" s="14" t="s">
         <v>129</v>
       </c>
@@ -8270,11 +8390,11 @@
       <c r="C41" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
       <c r="G41" s="14" t="s">
         <v>133</v>
       </c>
@@ -8289,11 +8409,11 @@
       <c r="C42" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="33" t="s">
+      <c r="D42" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
       <c r="G42" s="14" t="s">
         <v>137</v>
       </c>
@@ -8308,11 +8428,11 @@
       <c r="C43" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
       <c r="G43" s="14" t="s">
         <v>141</v>
       </c>
@@ -8322,16 +8442,16 @@
         <v>6</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>142</v>
+        <v>220</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="D44" s="33" t="s">
-        <v>143</v>
-      </c>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
+        <v>194</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
       <c r="G44" s="14" t="s">
         <v>144</v>
       </c>
@@ -8346,23 +8466,23 @@
       <c r="C45" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
       <c r="G45" s="14" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="26"/>
-      <c r="B46" s="27"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="28"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="22"/>
     </row>
     <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
@@ -8371,10 +8491,10 @@
       <c r="B47" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D47" s="30"/>
+      <c r="D47" s="24"/>
       <c r="E47" s="12" t="s">
         <v>4</v>
       </c>
@@ -8385,71 +8505,83 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="C48" s="23"/>
-      <c r="D48" s="24"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="29"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
     </row>
-    <row r="49" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="C49" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="D49" s="21"/>
+    <row r="49" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="9"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="25"/>
+      <c r="D49" s="25"/>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
-      <c r="C50" s="23"/>
-      <c r="D50" s="24"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="29"/>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="24"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="29"/>
       <c r="E51" s="11"/>
       <c r="F51" s="11"/>
       <c r="G51" s="11"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="24"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="29"/>
       <c r="E52" s="11"/>
       <c r="F52" s="11"/>
       <c r="G52" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:D3"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D31:F31"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="D15:F15"/>
@@ -8466,32 +8598,14 @@
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="D26:F26"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:D3"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="D42:F42"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.25" footer="0.3"/>
@@ -8527,14 +8641,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="37" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="34"/>
+      <c r="D1" s="40"/>
       <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
@@ -8546,24 +8660,24 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34"/>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
     </row>
     <row r="4" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -8572,15 +8686,15 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
     </row>
     <row r="7" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -8588,15 +8702,15 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
     </row>
     <row r="9" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
@@ -8613,11 +8727,11 @@
       <c r="C10" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
       <c r="G10" s="6" t="s">
         <v>56</v>
       </c>
@@ -8626,13 +8740,13 @@
       <c r="A11" s="5"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="36"/>
-      <c r="F11" s="36"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
       <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7" ht="223.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8641,13 +8755,13 @@
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="D12" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
       <c r="G12" s="8" t="s">
         <v>150</v>
       </c>
@@ -8658,13 +8772,13 @@
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
+        <v>224</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>238</v>
+      </c>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
       <c r="G13" s="8" t="s">
         <v>151</v>
       </c>
@@ -8675,13 +8789,13 @@
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D14" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
       <c r="G14" s="8" t="s">
         <v>152</v>
       </c>
@@ -8690,9 +8804,9 @@
       <c r="A15" s="5"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
       <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8705,11 +8819,11 @@
       <c r="C16" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
       <c r="G16" s="6" t="s">
         <v>56</v>
       </c>
@@ -8718,9 +8832,9 @@
       <c r="A17" s="5"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
       <c r="G17" s="8"/>
     </row>
     <row r="18" spans="1:7" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8729,13 +8843,13 @@
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="D18" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
       <c r="G18" s="8" t="s">
         <v>153</v>
       </c>
@@ -8746,13 +8860,13 @@
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D19" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="D19" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
       <c r="G19" s="8" t="s">
         <v>154</v>
       </c>
@@ -8763,13 +8877,13 @@
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="36" t="s">
-        <v>163</v>
-      </c>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
+        <v>228</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
       <c r="G20" s="8" t="s">
         <v>154</v>
       </c>
@@ -8780,13 +8894,13 @@
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="D21" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
       <c r="G21" s="8" t="s">
         <v>68</v>
       </c>
@@ -8795,9 +8909,9 @@
       <c r="A22" s="5"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
       <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8810,11 +8924,11 @@
       <c r="C23" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="37" t="s">
+      <c r="D23" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
       <c r="G23" s="6" t="s">
         <v>56</v>
       </c>
@@ -8823,9 +8937,9 @@
       <c r="A24" s="5"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
       <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:7" ht="151.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -8834,13 +8948,13 @@
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D25" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="D25" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
       <c r="G25" s="8" t="s">
         <v>71</v>
       </c>
@@ -8851,13 +8965,13 @@
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="D26" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="D26" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="36"/>
-      <c r="F26" s="36"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
       <c r="G26" s="8" t="s">
         <v>74</v>
       </c>
@@ -8868,13 +8982,13 @@
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D27" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="D27" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
       <c r="G27" s="8" t="s">
         <v>77</v>
       </c>
@@ -8885,13 +8999,13 @@
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="D28" s="34" t="s">
         <v>164</v>
       </c>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
       <c r="G28" s="8" t="s">
         <v>155</v>
       </c>
@@ -8902,13 +9016,13 @@
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D29" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="D29" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
       <c r="G29" s="8" t="s">
         <v>81</v>
       </c>
@@ -8917,9 +9031,9 @@
       <c r="A30" s="5"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="36"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
       <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8932,11 +9046,11 @@
       <c r="C31" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="37" t="s">
+      <c r="D31" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
       <c r="G31" s="6" t="s">
         <v>56</v>
       </c>
@@ -8945,9 +9059,9 @@
       <c r="A32" s="5"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
       <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8956,13 +9070,13 @@
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D33" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="D33" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E33" s="36"/>
-      <c r="F33" s="36"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
       <c r="G33" s="8" t="s">
         <v>156</v>
       </c>
@@ -8973,13 +9087,13 @@
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D34" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="D34" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
       <c r="G34" s="8" t="s">
         <v>157</v>
       </c>
@@ -8990,13 +9104,13 @@
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="D35" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
       <c r="G35" s="8" t="s">
         <v>158</v>
       </c>
@@ -9007,18 +9121,18 @@
       <c r="C36" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="36" t="s">
+      <c r="D36" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
       <c r="G36" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>167</v>
+        <v>240</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -9031,11 +9145,11 @@
       <c r="C38" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="D38" s="37" t="s">
+      <c r="D38" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
+      <c r="E38" s="35"/>
+      <c r="F38" s="35"/>
       <c r="G38" s="6" t="s">
         <v>172</v>
       </c>
@@ -9050,11 +9164,11 @@
       <c r="C39" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D39" s="42" t="s">
+      <c r="D39" s="36" t="s">
         <v>174</v>
       </c>
-      <c r="E39" s="42"/>
-      <c r="F39" s="42"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
       <c r="G39" s="15" t="s">
         <v>175</v>
       </c>
@@ -9069,11 +9183,11 @@
       <c r="C40" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D40" s="42" t="s">
+      <c r="D40" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="E40" s="42"/>
-      <c r="F40" s="42"/>
+      <c r="E40" s="36"/>
+      <c r="F40" s="36"/>
       <c r="G40" s="15" t="s">
         <v>178</v>
       </c>
@@ -9088,11 +9202,11 @@
       <c r="C41" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D41" s="42" t="s">
+      <c r="D41" s="36" t="s">
         <v>180</v>
       </c>
-      <c r="E41" s="42"/>
-      <c r="F41" s="42"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="36"/>
       <c r="G41" s="15" t="s">
         <v>181</v>
       </c>
@@ -9107,11 +9221,11 @@
       <c r="C42" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="42" t="s">
+      <c r="D42" s="36" t="s">
         <v>183</v>
       </c>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
+      <c r="E42" s="36"/>
+      <c r="F42" s="36"/>
       <c r="G42" s="15" t="s">
         <v>184</v>
       </c>
@@ -9126,11 +9240,11 @@
       <c r="C43" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D43" s="42" t="s">
+      <c r="D43" s="36" t="s">
         <v>186</v>
       </c>
-      <c r="E43" s="42"/>
-      <c r="F43" s="42"/>
+      <c r="E43" s="36"/>
+      <c r="F43" s="36"/>
       <c r="G43" s="15" t="s">
         <v>187</v>
       </c>
@@ -9140,16 +9254,16 @@
         <v>6</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>188</v>
+        <v>241</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>198</v>
-      </c>
-      <c r="D44" s="42" t="s">
-        <v>189</v>
-      </c>
-      <c r="E44" s="42"/>
-      <c r="F44" s="42"/>
+        <v>197</v>
+      </c>
+      <c r="D44" s="36" t="s">
+        <v>242</v>
+      </c>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36"/>
       <c r="G44" s="15" t="s">
         <v>190</v>
       </c>
@@ -9164,23 +9278,23 @@
       <c r="C45" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D45" s="42" t="s">
+      <c r="D45" s="36" t="s">
         <v>192</v>
       </c>
-      <c r="E45" s="42"/>
-      <c r="F45" s="42"/>
+      <c r="E45" s="36"/>
+      <c r="F45" s="36"/>
       <c r="G45" s="15" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="39"/>
-      <c r="B46" s="40"/>
-      <c r="C46" s="40"/>
-      <c r="D46" s="40"/>
-      <c r="E46" s="40"/>
-      <c r="F46" s="40"/>
-      <c r="G46" s="41"/>
+      <c r="A46" s="37"/>
+      <c r="B46" s="38"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="39"/>
     </row>
     <row r="47" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
@@ -9189,10 +9303,10 @@
       <c r="B47" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="D47" s="30"/>
+      <c r="D47" s="24"/>
       <c r="E47" s="12" t="s">
         <v>96</v>
       </c>
@@ -9205,30 +9319,22 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="C48" s="23" t="s">
-        <v>194</v>
-      </c>
-      <c r="D48" s="24"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="29"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
     </row>
     <row r="49" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="C49" s="36" t="s">
-        <v>206</v>
-      </c>
-      <c r="D49" s="36"/>
+      <c r="A49" s="9"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="34"/>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -9236,8 +9342,8 @@
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
-      <c r="C50" s="23"/>
-      <c r="D50" s="24"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="29"/>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -9245,8 +9351,8 @@
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="24"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="29"/>
       <c r="E51" s="11"/>
       <c r="F51" s="11"/>
       <c r="G51" s="11"/>
@@ -9254,14 +9360,48 @@
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="24"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="29"/>
       <c r="E52" s="11"/>
       <c r="F52" s="11"/>
       <c r="G52" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="50">
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:D3"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="A46:G46"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="C50:D50"/>
@@ -9278,40 +9418,6 @@
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="D43:F43"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:D3"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A8:G8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.25" footer="0.3"/>

</xml_diff>